<commit_message>
docs(order-management): lock 24.11 scope — two self-seeded trigger events, one email per action, recipient fallback chain
</commit_message>
<xml_diff>
--- a/order_management/24.11-order-cancellation-email-notification/24.11 - Order Cancellation - Email Notification.xlsx
+++ b/order_management/24.11-order-cancellation-email-notification/24.11 - Order Cancellation - Email Notification.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +85,13 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +113,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -147,6 +170,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,7 +595,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>5 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 0 out of scope.</t>
+          <t>Scope locked 2026-07-03 (Step-1 gate complete). 5 to implement here, 0 covered elsewhere, 0 out of scope. Rider on 24.9/24.10 (same release, builds after them).</t>
         </is>
       </c>
     </row>
@@ -585,7 +617,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>This story adds an optional, default-checked "Send cancellation/refund email notification" checkbox to the (net-new) admin Order cancel/refund actions, with the send decision enforced server-side: checked sends the exhibitor an email, unchecked sends nothing. Re-verification against code confirms the two load-bearing primitives exist and are reusable: the template email pipeline (MailerService.sendFromTemplate over SendGrid, which also logs every send to notification_logs) and the recipient address (Order.billing_email plus the Company relation). What does NOT yet exist: there is no order cancel/refund endpoint anywhere (the entire Order Management API is net-new), and no order-cancellation/refund trigger_event slug or notification template is seeded — only ppl_subscription_canceled. A confirmed gating detail: the notification-template create endpoint rejects any notification_type with no matching trigger_event, so a trigger_event slug must be seeded before any template can even be authored. The toggle flag, backend enforcement, and unchecked-suppression are straightforwardly Deliverable on the net-new endpoints; the actual "email is sent" path is Partial because the specific trigger_event + template must still be seeded and the cancel/refund action itself must execute.</t>
+          <t>Default-true send_notification toggle on cancel/refund, enforced server-side; ALL 5 rows Deliverable (24.11-c upgraded — artifacts story-owned per D2). D1: two slugs (order_canceled/order_refunded), one email per action. D3: billing_email -&gt; Company contact -&gt; skip+log. SBE-671 merged (caveat retired); known-issue #21 accepted risk.</t>
         </is>
       </c>
     </row>
@@ -610,7 +642,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -620,7 +652,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -661,7 +693,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete)</t>
         </is>
       </c>
     </row>
@@ -787,7 +819,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -819,17 +851,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The cancel/refund endpoints are net-new (no order controller exists; ppl-order is unrelated PPL-leads work), but adding a boolean field (e.g. send_notification) to their request DTO is trivial built-in NestJS/class-validator work, and OrderStatus already has canceled/refunded values to write. The UI checkbox is frontend, enabled by the flag.</t>
+          <t>CONFIRMED 2026-07-03. send_notification already provisioned in both owning DTOs (locked at the 24.9/24.10 gates, default true). Greps zero on dev (no collision). Evidence half-stale fix: orders module IS live (24.1-24.4) but has no cancel/refund route — routes are 24.9/24.10's same-release deliverables.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>no Order cancel/refund controller exists (only admin/ppl-order/ppl-order.controller.ts @Controller('ppl-orders'), PPL-leads); OrderStatus enum has canceled+refunded at admin-backend-api/prisma/schema.prisma; boolean DTO pattern at admin-backend-api/src/admin/product-management/dto/product-create.dto.ts:335+</t>
+          <t>admin orders.controller.ts:41 (module live, no cancel/refund route); grep send_notification = 0; product-create.dto.ts:329-372 (boolean-DTO precedent); OrderStatus canceled/refunded schema:426-427</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Cancel/refund action endpoints are themselves net-new within this same Order Management epic; this story's flag rides on them.</t>
+          <t>Rides 24.10 (SBE-1134) cancel DTO + 24.9 (SBE-1133) refund DTO — same release, build first</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -849,7 +881,7 @@
       </c>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable (flag already in owners’ locked DTO shapes).</t>
         </is>
       </c>
     </row>
@@ -881,12 +913,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Default-true is a one-line DTO default on the new boolean (@IsBoolean plus default true). Toggle is purely frontend; nothing in the codebase blocks it.</t>
+          <t>CONFIRMED 2026-07-03. One line per DTO: @IsBoolean() @IsOptional() send_notification?: boolean = true, default documented in ApiProperty. Contract: omitted/true =&gt; send; false =&gt; don't. Toggle UI is frontend.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>@IsBoolean DTO defaults used throughout, e.g. admin-backend-api/src/admin/product-management/dto/product-create.dto.ts:335,344,368; no order DTO exists yet</t>
+          <t>product-create.dto.ts:329-372 (boolean + default precedent)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -907,7 +939,7 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -924,7 +956,7 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -939,17 +971,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The send mechanism is fully built and reusable (MailerService.sendFromTemplate resolves an active EMAIL template by notification_type, HTML-escapes/substitutes tokens, wraps in the user layout, sends via SendGrid, and records a notification_logs row), and the recipient address is available (Order.billing_email plus Company relation). What is missing: NO order-cancellation/refund trigger_event slug or notification template is seeded (only ppl_subscription_canceled exists). Confirmed gate: the notification-template create endpoint rejects any notification_type with no matching trigger_event, so a trigger_event slug must be seeded before the template can be authored. The email can only fire once the net-new cancel/refund action runs.</t>
+          <t>CONFIRMED 2026-07-03 — upgraded Partial -&gt; Deliverable. Dispatch primitive live: sendFromTemplate (mailer.service.ts:192; resolution :198-204; send :235; notification_logs :242; non-throwing). Missing artifacts became STORY-OWNED under D2 (24.11 seeds 2 trigger_events w/ placeholder sets + 2 templates w/ TEMPLATE_META; template create validates per trigger, notification-template.service.ts:241/:448). DECIDED D1: order_canceled / order_refunded (names TBC vs catalogue), ONE EMAIL PER ACTION — cancel sends order_canceled (optional refund tokens); standalone refund sends order_refunded; never both. Known-issue #21 (custom shadows predefined) = accepted risk; fix ships with E&amp;S scheduling. SBE-671 verified MERGED (PR #426) — unmerged-branch caveat retired.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/common/services/mailer.service.ts:191-254 (sendFromTemplate, with notification_logs write at :241); trigger-event.seeder.ts slugs are ppl_subscription_canceled(:91), ppl_order_confirmation(:78), booth_order_confirmation(:216), ppl_product_order_payment(:191) — none for order cancel/refund; notification-template create rejects unknown notification_type (admin-backend-api/src/admin/notification-template/notification-template.controller.ts:216); Order.billing_email at admin-backend-api/prisma/schema.prisma:1563</t>
+          <t>mailer.service.ts:192/:198-204/:235/:242; trigger-event.seeder.ts 26 slugs (none cancel/refund; nearest ppl_subscription_canceled :104); notification-template.seeder.ts 24 templates + META guard :856-875; origin/dev..origin/feature/SBE-671 = 0 (2026-07-03)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>A cancellation/refund trigger_event slug (notification_type) plus matching seeded email template is owned by the Email &amp; SMS Management epic; the cancel/refund write-path is net-new in this epic.</t>
+          <t>Dispatch call sites live in 24.9/24.10 services — same release, build first</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -969,7 +1001,7 @@
       </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: upgraded Partial -&gt; Deliverable; D1 + D2 recorded.</t>
         </is>
       </c>
     </row>
@@ -1001,12 +1033,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Simple conditional in the net-new cancel/refund handler: only call MailerService.sendFromTemplate when the flag is true. The send is a single explicit call site, so gating it is trivial; no infrastructure gap.</t>
+          <t>CONFIRMED 2026-07-03. Exactly one send path to gate: the conditional sendFromTemplate call in each handler (sole send inside = sendMail :235). No background/queued email path exists for orders (worker mailer = 24.15's future cron leg only); no cancellation triggers exist for anything else to react to.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>mailer.service.ts:234 (sendMail invoked inside sendFromTemplate) is the sole send call site; no order handler exists yet to host the conditional</t>
+          <t>mailer.service.ts:235 (sole send call site); consolidation C4</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1027,7 +1059,7 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1091,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Enforcement is achieved by having the server read the validated flag and conditionally invoke the mailer inside the cancel/refund service; the client never sends email directly. Standard within existing service/controller patterns where all send calls are server-owned.</t>
+          <t>CONFIRMED 2026-07-03. All template sends server-owned via sendFromTemplate; no client-side send path. Enforcement = validated DTO flag read in the cancel/refund service. AGREED SHAPE: dispatch AFTER the $transaction commits (non-throwing mailer =&gt; failed email can't fail the action; rolled-back action never emailed); notification_logs = send audit; 24.9-h/24.10-i audit note captures the flag value. DECIDED D3 (applies with 24.11-c): recipient fallback chain Order.billing_email -&gt; Company contact email -&gt; skip + log (billing_email nullable String?, schema:1564); missing email never blocks the action.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>all template sends are server-side via mailer.service.ts:191 sendFromTemplate; no client-side email path exists in the codebase</t>
+          <t>mailer.service.ts:192 (server-owned), :208-210 (non-throwing); schema:1564 (billing_email String?)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1085,7 +1117,7 @@
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate locked 2026-07-03: Deliverable; post-commit dispatch + D3 fallback chain recorded.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1158,7 +1190,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Cancellation email behavior: send_notification (default true) toggles whether the exhibitor is emailed a cancellation notice; backend decides whether to send.</t>
+          <t>send_notification (default true) toggles the order_canceled email (token set incl. optional refund fields); dispatch post-commit via admin sendFromTemplate; recipient = D3 fallback chain.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1168,7 +1200,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>24.10 (owner — cancel execution), 24.12 (inventory release) — no separate route — reuses 24.10's cancel endpoint (send_notification flag).</t>
+          <t>24.10 (owner) — no separate route</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1217,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Refund email behavior: send_notification (default true) toggles whether the exhibitor is emailed a refund notice; backend decides whether to send.</t>
+          <t>send_notification (default true) toggles the order_refunded email; dispatch post-commit; one-email-per-action: never double-sends with cancel.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1195,7 +1227,34 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>24.9 (owner — refund execution), 24.6 — no separate route — reuses 24.9's refunds endpoint (send_notification flag).</t>
+          <t>24.9 (owner) — no separate route</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Seeders (admin)</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>2 trigger_events (order_canceled, order_refunded — names TBC vs catalogue) with declared placeholder sets + 2 EMAIL templates with TEMPLATE_META entries. Story-owned per D2.</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>24.11-c</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Naming consistency with the Email &amp; SMS catalogue (managed there, owned here)</t>
         </is>
       </c>
     </row>
@@ -1210,54 +1269,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Should cancellation and refund use one shared notification template or two distinct trigger_event slugs/templates? The spec frames a single combined checkbox ("Send cancellation/refund email notification"), but cancel and refund are distinct backend actions whose email content likely differs — this content/taxonomy decision is unresolved by the spec.</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>OPEN — for team discussion</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): (pending) leaning toward two distinct trigger_event slugs/templates (one for cancellation, one for refund) so each email carries action-appropriate content; the single combined checkbox can still drive both. To be confirmed with the team (owner: Email &amp; SMS Management epic) before any seeding.</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Register empty — gate locked 2026-07-03</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr"/>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Shared-vs-distinct template question RESOLVED: D1 two slugs (order_canceled/order_refunded), one email per action; D2 24.11 seeds its own artifacts (ownership rule: flows own templates, E&amp;S epic manages); D3 recipient chain billing_email -&gt; Company contact -&gt; skip+log.</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr"/>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>All 5 rows Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1298,19 +1387,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>A seeded cancellation/refund trigger_event slug (notification_type) and matching active EMAIL notification template for MailerService.sendFromTemplate to resolve. The trigger_event must exist first because the notification-template create endpoint rejects unknown notification_type values.</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>24.11-c</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Email &amp; SMS Management epic (owns notification_template / trigger_event taxonomy and seeders)</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Cancel/refund routes + DTOs (flag already in their locked shapes)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>24.11-a…e</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>24.10 (SBE-1134) / 24.9 (SBE-1133) — same release, build first</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Email &amp; SMS epic (informational, NOT a dependency): SBE-671 merged to dev (PR #426, verified 2026-07-03); 24.11 owns its slugs/templates per the 2026-07-03 ownership rule; E&amp;S manages the system + ships the #21 shadowing fix with scheduling</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Email &amp; SMS epic (management only)</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1345,146 +1451,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Implementation</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Not yet implemented — analysis/feasibility stage only; no branch or SBE ticket cut yet. Extended tracking format applied; per-requirement build status is ◻ Not started.</t>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03; scope + 3 decisions locked (D1 two slugs / one email per action; D2 story-owned seeding; D3 recipient fallback chain). Release model: all remaining OM stories ship together.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Branch / PR</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.11-a</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — send_notification boolean flag on the (net-new) cancel/refund request DTOs.</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>SBE-1135 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.11-b</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — default-checked/default-true behavior for the flag (DTO default; toggle is frontend).</t>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.11-c</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — checked → exhibitor cancellation/refund email sent; send path Partial (needs trigger_event slug + template seeded, then MailerService.sendFromTemplate dispatch).</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.11-d</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — unchecked → no automated email sent (conditional dispatch).</t>
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Remaining — 24.11-e</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — server-side enforcement of the notification choice inside the cancel/refund service.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Open decision — cancel/refund templates</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>One shared notification template vs two distinct trigger_event slugs/templates for cancellation vs refund. Current direction (2026-07-01): pending; leaning toward two distinct templates. Owner: Email &amp; SMS Management epic.</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Dependency — 24.10</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>POST /api/v1/orders/:id/cancel cancel action endpoint (net-new in this Order Management epic); 24.11 flag rides on it.</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>24.11-a/b/c/d/e — conditional dispatch in 24.9/24.10 services + 2 seeded trigger_events + 2 templates + fallback chain; post-commit dispatch shape</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Dependency — 24.9</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>POST /api/v1/orders/:id/refunds refund action endpoint (net-new in this Order Management epic); 24.11 flag rides on it.</t>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Remaining</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>All confirmed scope unbuilt</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Dependency — Email &amp; SMS Management epic</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>Seeded cancellation/refund trigger_event slug (notification_type) + matching active EMAIL notification template; needed for 24.11-c (create endpoint rejects unknown notification_type).</t>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Not ready — see Open Questions</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>none — register empty</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>24.9/24.10 routes — same release, build first; no true external dependency</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Out of API scope</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Front-end wiring — the checkbox UI element and its default-checked state.</t>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Checkbox UI + default-checked rendering (frontend)</t>
         </is>
       </c>
     </row>

</xml_diff>